<commit_message>
Tests sort of work but don't converge
</commit_message>
<xml_diff>
--- a/test_data/icpms_test/synthetic_data_2025_04_21_simple.xlsx
+++ b/test_data/icpms_test/synthetic_data_2025_04_21_simple.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Daven/Projects/Sparrow/Labs/Sparrow-CU-TRaIL/test_data/icpms_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1481C52F-EB08-874E-95C5-26847841FAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBC3914-0975-274B-8BDC-D88BCA19CB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="3080" windowWidth="25880" windowHeight="16940" xr2:uid="{B2FFEE73-7653-EB43-8267-ECB1A9954BEC}"/>
   </bookViews>
@@ -244,9 +244,6 @@
   </si>
   <si>
     <t>4He</t>
-  </si>
-  <si>
-    <t>4 He err</t>
   </si>
   <si>
     <t>238U</t>
@@ -420,6 +417,9 @@
       </rPr>
       <t>}</t>
     </r>
+  </si>
+  <si>
+    <t>4He err</t>
   </si>
 </sst>
 </file>
@@ -1026,25 +1026,25 @@
         <v>68</v>
       </c>
       <c r="L1" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="M1" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="N1" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="O1" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="Q1" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="R1" s="17" t="s">
         <v>74</v>
-      </c>
-      <c r="R1" s="17" t="s">
-        <v>75</v>
       </c>
       <c r="S1" s="13"/>
       <c r="T1" s="13" t="s">
@@ -3919,7 +3919,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3955,7 +3955,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -3977,12 +3977,12 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="18" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
         <v>66</v>
@@ -3990,12 +3990,12 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" t="s">
         <v>66</v>
@@ -4003,12 +4003,12 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B20" t="s">
         <v>66</v>
@@ -4016,7 +4016,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -4060,7 +4060,7 @@
         <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -4131,7 +4131,7 @@
         <v>51</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:2">

</xml_diff>